<commit_message>
continued work on random forests
</commit_message>
<xml_diff>
--- a/datasets/data_output_a.xlsx
+++ b/datasets/data_output_a.xlsx
@@ -1643,13 +1643,13 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -2634,7 +2634,7 @@
         <v>149</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="4" t="s">
         <v>150</v>
       </c>
@@ -3538,7 +3538,7 @@
         <v>155</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="4" t="s">
         <v>162</v>
       </c>
@@ -3990,7 +3990,7 @@
         <v>155</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="4" t="s">
         <v>167</v>
       </c>
@@ -4442,7 +4442,7 @@
         <v>155</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="4" t="s">
         <v>171</v>
       </c>
@@ -4894,7 +4894,7 @@
         <v>155</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="4" t="s">
         <v>176</v>
       </c>
@@ -5346,7 +5346,7 @@
         <v>155</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="4" t="s">
         <v>180</v>
       </c>
@@ -5798,7 +5798,7 @@
         <v>155</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="4" t="s">
         <v>185</v>
       </c>
@@ -6250,7 +6250,7 @@
         <v>155</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="4" t="s">
         <v>190</v>
       </c>
@@ -6702,7 +6702,7 @@
         <v>155</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="4" t="s">
         <v>194</v>
       </c>
@@ -7606,7 +7606,7 @@
         <v>155</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="4" t="s">
         <v>201</v>
       </c>

</xml_diff>